<commit_message>
Updated for 7th September
</commit_message>
<xml_diff>
--- a/12601870.xlsx
+++ b/12601870.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/370a177e9e66eb08/Documents/GitHub/Daily-Activity-tracker-CAP776-Python/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="365" documentId="13_ncr:1_{1A11B410-6228-4EFB-ADF5-2519D16142E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C6071D77-6F8B-43C2-8862-E0F42BBAFBB5}"/>
+  <xr:revisionPtr revIDLastSave="377" documentId="13_ncr:1_{1A11B410-6228-4EFB-ADF5-2519D16142E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EC246AA5-2115-4035-B4A3-373CE937FB4C}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="92">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -310,6 +310,9 @@
   </si>
   <si>
     <t>Today I started prepairing for the CA</t>
+  </si>
+  <si>
+    <t>Today I practiced SQL for 6 straight hours.</t>
   </si>
 </sst>
 </file>
@@ -2425,27 +2428,51 @@
         <v>90</v>
       </c>
     </row>
-    <row r="34" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A34" s="18"/>
-      <c r="B34" s="19"/>
-      <c r="C34" s="19"/>
-      <c r="D34" s="19"/>
-      <c r="E34" s="19"/>
-      <c r="F34" s="19"/>
-      <c r="G34" s="19"/>
-      <c r="H34" s="19"/>
-      <c r="I34" s="20" t="str">
+    <row r="34" spans="1:14" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A34" s="18">
+        <v>46272</v>
+      </c>
+      <c r="B34" s="19">
+        <v>420</v>
+      </c>
+      <c r="C34" s="19">
+        <v>36</v>
+      </c>
+      <c r="D34" s="19">
+        <v>360</v>
+      </c>
+      <c r="E34" s="19">
+        <v>180</v>
+      </c>
+      <c r="F34" s="19">
+        <v>150</v>
+      </c>
+      <c r="G34" s="19">
+        <v>3</v>
+      </c>
+      <c r="H34" s="19">
+        <v>200</v>
+      </c>
+      <c r="I34" s="20">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J34" s="20" t="str">
+        <v>1346</v>
+      </c>
+      <c r="J34" s="20">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K34" s="21"/>
-      <c r="L34" s="21"/>
-      <c r="M34" s="21"/>
-      <c r="N34" s="22"/>
+        <v>94</v>
+      </c>
+      <c r="K34" s="21" t="s">
+        <v>48</v>
+      </c>
+      <c r="L34" s="21" t="s">
+        <v>56</v>
+      </c>
+      <c r="M34" s="21" t="s">
+        <v>68</v>
+      </c>
+      <c r="N34" s="22" t="s">
+        <v>91</v>
+      </c>
     </row>
     <row r="35" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A35" s="18"/>

</xml_diff>

<commit_message>
Updated for 8th August
</commit_message>
<xml_diff>
--- a/12601870.xlsx
+++ b/12601870.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/370a177e9e66eb08/Documents/GitHub/Daily-Activity-tracker-CAP776-Python/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="377" documentId="13_ncr:1_{1A11B410-6228-4EFB-ADF5-2519D16142E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EC246AA5-2115-4035-B4A3-373CE937FB4C}"/>
+  <xr:revisionPtr revIDLastSave="389" documentId="13_ncr:1_{1A11B410-6228-4EFB-ADF5-2519D16142E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DF3B356E-81EB-4758-9AE4-05CD8DA7E4FF}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="93">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -313,6 +313,9 @@
   </si>
   <si>
     <t>Today I practiced SQL for 6 straight hours.</t>
+  </si>
+  <si>
+    <t>After Completing Half of Today's CA I started prepairing for Tomorrow's CA.</t>
   </si>
 </sst>
 </file>
@@ -2474,27 +2477,51 @@
         <v>91</v>
       </c>
     </row>
-    <row r="35" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A35" s="18"/>
-      <c r="B35" s="19"/>
-      <c r="C35" s="19"/>
-      <c r="D35" s="19"/>
-      <c r="E35" s="19"/>
-      <c r="F35" s="19"/>
-      <c r="G35" s="19"/>
-      <c r="H35" s="19"/>
-      <c r="I35" s="20" t="str">
+    <row r="35" spans="1:14" ht="62.4" x14ac:dyDescent="0.3">
+      <c r="A35" s="18">
+        <v>46273</v>
+      </c>
+      <c r="B35" s="19">
+        <v>280</v>
+      </c>
+      <c r="C35" s="19">
+        <v>30</v>
+      </c>
+      <c r="D35" s="19">
+        <v>120</v>
+      </c>
+      <c r="E35" s="19">
+        <v>0</v>
+      </c>
+      <c r="F35" s="19">
+        <v>250</v>
+      </c>
+      <c r="G35" s="19">
+        <v>5</v>
+      </c>
+      <c r="H35" s="19">
+        <v>0</v>
+      </c>
+      <c r="I35" s="20">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J35" s="20" t="str">
+        <v>680</v>
+      </c>
+      <c r="J35" s="20">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K35" s="21"/>
-      <c r="L35" s="21"/>
-      <c r="M35" s="21"/>
-      <c r="N35" s="22"/>
+        <v>760</v>
+      </c>
+      <c r="K35" s="21" t="s">
+        <v>60</v>
+      </c>
+      <c r="L35" s="21" t="s">
+        <v>61</v>
+      </c>
+      <c r="M35" s="21" t="s">
+        <v>54</v>
+      </c>
+      <c r="N35" s="22" t="s">
+        <v>92</v>
+      </c>
     </row>
     <row r="36" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A36" s="18"/>

</xml_diff>

<commit_message>
Updated for 9th August
</commit_message>
<xml_diff>
--- a/12601870.xlsx
+++ b/12601870.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/370a177e9e66eb08/Documents/GitHub/Daily-Activity-tracker-CAP776-Python/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="389" documentId="13_ncr:1_{1A11B410-6228-4EFB-ADF5-2519D16142E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DF3B356E-81EB-4758-9AE4-05CD8DA7E4FF}"/>
+  <xr:revisionPtr revIDLastSave="403" documentId="13_ncr:1_{1A11B410-6228-4EFB-ADF5-2519D16142E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FE845184-DCA0-41D2-91A5-FA2CED236021}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="94">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -316,6 +316,9 @@
   </si>
   <si>
     <t>After Completing Half of Today's CA I started prepairing for Tomorrow's CA.</t>
+  </si>
+  <si>
+    <t>Today I completed 2 Ca's Now I will just rest.</t>
   </si>
 </sst>
 </file>
@@ -2523,27 +2526,51 @@
         <v>92</v>
       </c>
     </row>
-    <row r="36" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A36" s="18"/>
-      <c r="B36" s="19"/>
-      <c r="C36" s="19"/>
-      <c r="D36" s="19"/>
-      <c r="E36" s="19"/>
-      <c r="F36" s="19"/>
-      <c r="G36" s="19"/>
-      <c r="H36" s="19"/>
-      <c r="I36" s="20" t="str">
+    <row r="36" spans="1:14" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A36" s="18">
+        <v>46274</v>
+      </c>
+      <c r="B36" s="19">
+        <v>360</v>
+      </c>
+      <c r="C36" s="19">
+        <v>45</v>
+      </c>
+      <c r="D36" s="19">
+        <v>25</v>
+      </c>
+      <c r="E36" s="19">
+        <v>10</v>
+      </c>
+      <c r="F36" s="19">
+        <v>300</v>
+      </c>
+      <c r="G36" s="19">
+        <v>6</v>
+      </c>
+      <c r="H36" s="19">
+        <v>0</v>
+      </c>
+      <c r="I36" s="20">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J36" s="20" t="str">
+        <v>740</v>
+      </c>
+      <c r="J36" s="20">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K36" s="21"/>
-      <c r="L36" s="21"/>
-      <c r="M36" s="21"/>
-      <c r="N36" s="22"/>
+        <v>700</v>
+      </c>
+      <c r="K36" s="21" t="s">
+        <v>56</v>
+      </c>
+      <c r="L36" s="21" t="s">
+        <v>56</v>
+      </c>
+      <c r="M36" s="21" t="s">
+        <v>54</v>
+      </c>
+      <c r="N36" s="22" t="s">
+        <v>93</v>
+      </c>
     </row>
     <row r="37" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A37" s="18"/>

</xml_diff>

<commit_message>
Updated for 10th September
</commit_message>
<xml_diff>
--- a/12601870.xlsx
+++ b/12601870.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/370a177e9e66eb08/Documents/GitHub/Daily-Activity-tracker-CAP776-Python/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="403" documentId="13_ncr:1_{1A11B410-6228-4EFB-ADF5-2519D16142E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FE845184-DCA0-41D2-91A5-FA2CED236021}"/>
+  <xr:revisionPtr revIDLastSave="415" documentId="13_ncr:1_{1A11B410-6228-4EFB-ADF5-2519D16142E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{98B1126D-8876-434D-976A-A7B6BFBF1322}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="95">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -319,6 +319,9 @@
   </si>
   <si>
     <t>Today I completed 2 Ca's Now I will just rest.</t>
+  </si>
+  <si>
+    <t>Today we had Fresher's party .</t>
   </si>
 </sst>
 </file>
@@ -2572,27 +2575,51 @@
         <v>93</v>
       </c>
     </row>
-    <row r="37" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A37" s="18"/>
-      <c r="B37" s="19"/>
-      <c r="C37" s="19"/>
-      <c r="D37" s="19"/>
-      <c r="E37" s="19"/>
-      <c r="F37" s="19"/>
-      <c r="G37" s="19"/>
-      <c r="H37" s="19"/>
-      <c r="I37" s="20" t="str">
+    <row r="37" spans="1:14" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A37" s="18">
+        <v>46275</v>
+      </c>
+      <c r="B37" s="19">
+        <v>540</v>
+      </c>
+      <c r="C37" s="19">
+        <v>60</v>
+      </c>
+      <c r="D37" s="19">
+        <v>0</v>
+      </c>
+      <c r="E37" s="19">
+        <v>0</v>
+      </c>
+      <c r="F37" s="19">
+        <v>200</v>
+      </c>
+      <c r="G37" s="19">
+        <v>4</v>
+      </c>
+      <c r="H37" s="19">
+        <v>0</v>
+      </c>
+      <c r="I37" s="20">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J37" s="20" t="str">
+        <v>800</v>
+      </c>
+      <c r="J37" s="20">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K37" s="21"/>
-      <c r="L37" s="21"/>
-      <c r="M37" s="21"/>
-      <c r="N37" s="22"/>
+        <v>640</v>
+      </c>
+      <c r="K37" s="21" t="s">
+        <v>63</v>
+      </c>
+      <c r="L37" s="21" t="s">
+        <v>57</v>
+      </c>
+      <c r="M37" s="21" t="s">
+        <v>64</v>
+      </c>
+      <c r="N37" s="22" t="s">
+        <v>94</v>
+      </c>
     </row>
     <row r="38" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A38" s="18"/>

</xml_diff>

<commit_message>
Updated for 11th September
</commit_message>
<xml_diff>
--- a/12601870.xlsx
+++ b/12601870.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/370a177e9e66eb08/Documents/GitHub/Daily-Activity-tracker-CAP776-Python/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="415" documentId="13_ncr:1_{1A11B410-6228-4EFB-ADF5-2519D16142E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{98B1126D-8876-434D-976A-A7B6BFBF1322}"/>
+  <xr:revisionPtr revIDLastSave="427" documentId="13_ncr:1_{1A11B410-6228-4EFB-ADF5-2519D16142E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4CBCBE0D-4B7C-43F4-A609-C4A96473B9F0}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="96">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -322,6 +322,9 @@
   </si>
   <si>
     <t>Today we had Fresher's party .</t>
+  </si>
+  <si>
+    <t>Today I encountererd Problem due to the mars paltform</t>
   </si>
 </sst>
 </file>
@@ -2621,27 +2624,51 @@
         <v>94</v>
       </c>
     </row>
-    <row r="38" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A38" s="18"/>
-      <c r="B38" s="19"/>
-      <c r="C38" s="19"/>
-      <c r="D38" s="19"/>
-      <c r="E38" s="19"/>
-      <c r="F38" s="19"/>
-      <c r="G38" s="19"/>
-      <c r="H38" s="19"/>
-      <c r="I38" s="20" t="str">
+    <row r="38" spans="1:14" ht="46.8" x14ac:dyDescent="0.3">
+      <c r="A38" s="18">
+        <v>46276</v>
+      </c>
+      <c r="B38" s="19">
+        <v>360</v>
+      </c>
+      <c r="C38" s="19">
+        <v>39</v>
+      </c>
+      <c r="D38" s="19">
+        <v>120</v>
+      </c>
+      <c r="E38" s="19">
+        <v>45</v>
+      </c>
+      <c r="F38" s="19">
+        <v>150</v>
+      </c>
+      <c r="G38" s="19">
+        <v>3</v>
+      </c>
+      <c r="H38" s="19">
+        <v>0</v>
+      </c>
+      <c r="I38" s="20">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J38" s="20" t="str">
+        <v>714</v>
+      </c>
+      <c r="J38" s="20">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K38" s="21"/>
-      <c r="L38" s="21"/>
-      <c r="M38" s="21"/>
-      <c r="N38" s="22"/>
+        <v>726</v>
+      </c>
+      <c r="K38" s="21" t="s">
+        <v>48</v>
+      </c>
+      <c r="L38" s="21" t="s">
+        <v>49</v>
+      </c>
+      <c r="M38" s="21" t="s">
+        <v>68</v>
+      </c>
+      <c r="N38" s="22" t="s">
+        <v>95</v>
+      </c>
     </row>
     <row r="39" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A39" s="18"/>

</xml_diff>

<commit_message>
Updated for 13th September
</commit_message>
<xml_diff>
--- a/12601870.xlsx
+++ b/12601870.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/370a177e9e66eb08/Documents/GitHub/Daily-Activity-tracker-CAP776-Python/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="427" documentId="13_ncr:1_{1A11B410-6228-4EFB-ADF5-2519D16142E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4CBCBE0D-4B7C-43F4-A609-C4A96473B9F0}"/>
+  <xr:revisionPtr revIDLastSave="440" documentId="13_ncr:1_{1A11B410-6228-4EFB-ADF5-2519D16142E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BC873EB7-ADC6-40C0-A88D-8282DB2FDDB7}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="97">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -325,6 +325,9 @@
   </si>
   <si>
     <t>Today I encountererd Problem due to the mars paltform</t>
+  </si>
+  <si>
+    <t>Today I practiced Python for the upcoming CA.</t>
   </si>
 </sst>
 </file>
@@ -2670,27 +2673,51 @@
         <v>95</v>
       </c>
     </row>
-    <row r="39" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A39" s="18"/>
-      <c r="B39" s="19"/>
-      <c r="C39" s="19"/>
-      <c r="D39" s="19"/>
-      <c r="E39" s="19"/>
-      <c r="F39" s="19"/>
-      <c r="G39" s="19"/>
-      <c r="H39" s="19"/>
-      <c r="I39" s="20" t="str">
+    <row r="39" spans="1:14" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A39" s="18">
+        <v>46278</v>
+      </c>
+      <c r="B39" s="19">
+        <v>420</v>
+      </c>
+      <c r="C39" s="19">
+        <v>90</v>
+      </c>
+      <c r="D39" s="19">
+        <v>180</v>
+      </c>
+      <c r="E39" s="19">
+        <v>60</v>
+      </c>
+      <c r="F39" s="19">
+        <v>0</v>
+      </c>
+      <c r="G39" s="19">
+        <v>0</v>
+      </c>
+      <c r="H39" s="19">
+        <v>240</v>
+      </c>
+      <c r="I39" s="20">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J39" s="20" t="str">
+        <v>990</v>
+      </c>
+      <c r="J39" s="20">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K39" s="21"/>
-      <c r="L39" s="21"/>
-      <c r="M39" s="21"/>
-      <c r="N39" s="22"/>
+        <v>450</v>
+      </c>
+      <c r="K39" s="21" t="s">
+        <v>48</v>
+      </c>
+      <c r="L39" s="21" t="s">
+        <v>70</v>
+      </c>
+      <c r="M39" s="21" t="s">
+        <v>68</v>
+      </c>
+      <c r="N39" s="22" t="s">
+        <v>96</v>
+      </c>
     </row>
     <row r="40" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A40" s="18"/>

</xml_diff>

<commit_message>
Updated for 15th September
</commit_message>
<xml_diff>
--- a/12601870.xlsx
+++ b/12601870.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/370a177e9e66eb08/Documents/GitHub/Daily-Activity-tracker-CAP776-Python/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="440" documentId="13_ncr:1_{1A11B410-6228-4EFB-ADF5-2519D16142E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BC873EB7-ADC6-40C0-A88D-8282DB2FDDB7}"/>
+  <xr:revisionPtr revIDLastSave="453" documentId="13_ncr:1_{1A11B410-6228-4EFB-ADF5-2519D16142E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AC7BD706-4ABE-4C53-8368-114B46856706}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="98">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -328,6 +328,9 @@
   </si>
   <si>
     <t>Today I practiced Python for the upcoming CA.</t>
+  </si>
+  <si>
+    <t>Python CA done.</t>
   </si>
 </sst>
 </file>
@@ -2720,26 +2723,50 @@
       </c>
     </row>
     <row r="40" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A40" s="18"/>
-      <c r="B40" s="19"/>
-      <c r="C40" s="19"/>
-      <c r="D40" s="19"/>
-      <c r="E40" s="19"/>
-      <c r="F40" s="19"/>
-      <c r="G40" s="19"/>
-      <c r="H40" s="19"/>
-      <c r="I40" s="20" t="str">
+      <c r="A40" s="18">
+        <v>46280</v>
+      </c>
+      <c r="B40" s="19">
+        <v>423</v>
+      </c>
+      <c r="C40" s="19">
+        <v>125</v>
+      </c>
+      <c r="D40" s="19">
+        <v>320</v>
+      </c>
+      <c r="E40" s="19">
+        <v>145</v>
+      </c>
+      <c r="F40" s="19">
+        <v>200</v>
+      </c>
+      <c r="G40" s="19">
+        <v>4</v>
+      </c>
+      <c r="H40" s="19">
+        <v>0</v>
+      </c>
+      <c r="I40" s="20">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J40" s="20" t="str">
+        <v>1213</v>
+      </c>
+      <c r="J40" s="20">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K40" s="21"/>
-      <c r="L40" s="21"/>
-      <c r="M40" s="21"/>
-      <c r="N40" s="22"/>
+        <v>227</v>
+      </c>
+      <c r="K40" s="21" t="s">
+        <v>56</v>
+      </c>
+      <c r="L40" s="21" t="s">
+        <v>49</v>
+      </c>
+      <c r="M40" s="21" t="s">
+        <v>68</v>
+      </c>
+      <c r="N40" s="22" t="s">
+        <v>97</v>
+      </c>
     </row>
     <row r="41" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A41" s="18"/>

</xml_diff>

<commit_message>
Updated for 16th September
</commit_message>
<xml_diff>
--- a/12601870.xlsx
+++ b/12601870.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/370a177e9e66eb08/Documents/GitHub/Daily-Activity-tracker-CAP776-Python/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="453" documentId="13_ncr:1_{1A11B410-6228-4EFB-ADF5-2519D16142E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AC7BD706-4ABE-4C53-8368-114B46856706}"/>
+  <xr:revisionPtr revIDLastSave="465" documentId="13_ncr:1_{1A11B410-6228-4EFB-ADF5-2519D16142E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E1291ACB-ECF7-4459-8DA3-15EA4735CC15}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="99">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -331,6 +331,9 @@
   </si>
   <si>
     <t>Python CA done.</t>
+  </si>
+  <si>
+    <t>Today the result of two Cas were declared.</t>
   </si>
 </sst>
 </file>
@@ -2768,27 +2771,51 @@
         <v>97</v>
       </c>
     </row>
-    <row r="41" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A41" s="18"/>
-      <c r="B41" s="19"/>
-      <c r="C41" s="19"/>
-      <c r="D41" s="19"/>
-      <c r="E41" s="19"/>
-      <c r="F41" s="19"/>
-      <c r="G41" s="19"/>
-      <c r="H41" s="19"/>
-      <c r="I41" s="20" t="str">
+    <row r="41" spans="1:14" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A41" s="18">
+        <v>46281</v>
+      </c>
+      <c r="B41" s="19">
+        <v>420</v>
+      </c>
+      <c r="C41" s="19">
+        <v>120</v>
+      </c>
+      <c r="D41" s="19">
+        <v>85</v>
+      </c>
+      <c r="E41" s="19">
+        <v>0</v>
+      </c>
+      <c r="F41" s="19">
+        <v>400</v>
+      </c>
+      <c r="G41" s="19">
+        <v>8</v>
+      </c>
+      <c r="H41" s="19">
+        <v>0</v>
+      </c>
+      <c r="I41" s="20">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J41" s="20" t="str">
+        <v>1025</v>
+      </c>
+      <c r="J41" s="20">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K41" s="21"/>
-      <c r="L41" s="21"/>
-      <c r="M41" s="21"/>
-      <c r="N41" s="22"/>
+        <v>415</v>
+      </c>
+      <c r="K41" s="21" t="s">
+        <v>60</v>
+      </c>
+      <c r="L41" s="21" t="s">
+        <v>61</v>
+      </c>
+      <c r="M41" s="21" t="s">
+        <v>54</v>
+      </c>
+      <c r="N41" s="22" t="s">
+        <v>98</v>
+      </c>
     </row>
     <row r="42" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A42" s="18"/>

</xml_diff>

<commit_message>
Updated for 17th September
</commit_message>
<xml_diff>
--- a/12601870.xlsx
+++ b/12601870.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/370a177e9e66eb08/Documents/GitHub/Daily-Activity-tracker-CAP776-Python/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="465" documentId="13_ncr:1_{1A11B410-6228-4EFB-ADF5-2519D16142E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E1291ACB-ECF7-4459-8DA3-15EA4735CC15}"/>
+  <xr:revisionPtr revIDLastSave="477" documentId="13_ncr:1_{1A11B410-6228-4EFB-ADF5-2519D16142E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F1F3A6BE-E622-4DFB-9BF9-C6D47C0C3760}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="200" uniqueCount="100">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -334,6 +334,9 @@
   </si>
   <si>
     <t>Today the result of two Cas were declared.</t>
+  </si>
+  <si>
+    <t>Today I'm Preparing for the Analytical CA.</t>
   </si>
 </sst>
 </file>
@@ -2817,27 +2820,51 @@
         <v>98</v>
       </c>
     </row>
-    <row r="42" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A42" s="18"/>
-      <c r="B42" s="19"/>
-      <c r="C42" s="19"/>
-      <c r="D42" s="19"/>
-      <c r="E42" s="19"/>
-      <c r="F42" s="19"/>
-      <c r="G42" s="19"/>
-      <c r="H42" s="19"/>
-      <c r="I42" s="20" t="str">
+    <row r="42" spans="1:14" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A42" s="18">
+        <v>46282</v>
+      </c>
+      <c r="B42" s="19">
+        <v>300</v>
+      </c>
+      <c r="C42" s="19">
+        <v>140</v>
+      </c>
+      <c r="D42" s="19">
+        <v>360</v>
+      </c>
+      <c r="E42" s="19">
+        <v>0</v>
+      </c>
+      <c r="F42" s="19">
+        <v>250</v>
+      </c>
+      <c r="G42" s="19">
+        <v>5</v>
+      </c>
+      <c r="H42" s="19">
+        <v>0</v>
+      </c>
+      <c r="I42" s="20">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J42" s="20" t="str">
+        <v>1050</v>
+      </c>
+      <c r="J42" s="20">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K42" s="21"/>
-      <c r="L42" s="21"/>
-      <c r="M42" s="21"/>
-      <c r="N42" s="22"/>
+        <v>390</v>
+      </c>
+      <c r="K42" s="21" t="s">
+        <v>60</v>
+      </c>
+      <c r="L42" s="21" t="s">
+        <v>70</v>
+      </c>
+      <c r="M42" s="21" t="s">
+        <v>54</v>
+      </c>
+      <c r="N42" s="22" t="s">
+        <v>99</v>
+      </c>
     </row>
     <row r="43" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A43" s="18"/>

</xml_diff>

<commit_message>
Updated for 18th September
</commit_message>
<xml_diff>
--- a/12601870.xlsx
+++ b/12601870.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/370a177e9e66eb08/Documents/GitHub/Daily-Activity-tracker-CAP776-Python/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="477" documentId="13_ncr:1_{1A11B410-6228-4EFB-ADF5-2519D16142E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F1F3A6BE-E622-4DFB-9BF9-C6D47C0C3760}"/>
+  <xr:revisionPtr revIDLastSave="489" documentId="13_ncr:1_{1A11B410-6228-4EFB-ADF5-2519D16142E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{46E49992-930F-4D05-BEB7-5079B99ADA1A}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="200" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="378" uniqueCount="101">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -337,6 +337,9 @@
   </si>
   <si>
     <t>Today I'm Preparing for the Analytical CA.</t>
+  </si>
+  <si>
+    <t>Preparation of Analytical CA is still going.</t>
   </si>
 </sst>
 </file>
@@ -2866,27 +2869,51 @@
         <v>99</v>
       </c>
     </row>
-    <row r="43" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A43" s="18"/>
-      <c r="B43" s="19"/>
-      <c r="C43" s="19"/>
-      <c r="D43" s="19"/>
-      <c r="E43" s="19"/>
-      <c r="F43" s="19"/>
-      <c r="G43" s="19"/>
-      <c r="H43" s="19"/>
-      <c r="I43" s="20" t="str">
+    <row r="43" spans="1:14" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A43" s="18">
+        <v>46283</v>
+      </c>
+      <c r="B43" s="19">
+        <v>420</v>
+      </c>
+      <c r="C43" s="19">
+        <v>120</v>
+      </c>
+      <c r="D43" s="19">
+        <v>360</v>
+      </c>
+      <c r="E43" s="19">
+        <v>0</v>
+      </c>
+      <c r="F43" s="19">
+        <v>250</v>
+      </c>
+      <c r="G43" s="19">
+        <v>5</v>
+      </c>
+      <c r="H43" s="19">
+        <v>0</v>
+      </c>
+      <c r="I43" s="20">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J43" s="20" t="str">
+        <v>1150</v>
+      </c>
+      <c r="J43" s="20">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K43" s="21"/>
-      <c r="L43" s="21"/>
-      <c r="M43" s="21"/>
-      <c r="N43" s="22"/>
+        <v>290</v>
+      </c>
+      <c r="K43" s="21" t="s">
+        <v>54</v>
+      </c>
+      <c r="L43" s="21" t="s">
+        <v>61</v>
+      </c>
+      <c r="M43" s="21" t="s">
+        <v>68</v>
+      </c>
+      <c r="N43" s="22" t="s">
+        <v>100</v>
+      </c>
     </row>
     <row r="44" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A44" s="18"/>

</xml_diff>